<commit_message>
trabajos con  los inventarios especificamente con el reporte de master
</commit_message>
<xml_diff>
--- a/bin/Debug/net9.0-windows/InventarioMaster.xlsx
+++ b/bin/Debug/net9.0-windows/InventarioMaster.xlsx
@@ -2165,7 +2165,7 @@
         <x:v>45849</x:v>
       </x:c>
       <x:c r="S2" s="3">
-        <x:v>45892.6204811458</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:19">
@@ -2218,7 +2218,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S3" s="3">
-        <x:v>45892.6204811458</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:19">
@@ -2271,7 +2271,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S4" s="3">
-        <x:v>45892.6204811458</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:19">
@@ -2324,7 +2324,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S5" s="3">
-        <x:v>45892.6204811458</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:19">
@@ -2377,7 +2377,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S6" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:19">
@@ -2430,7 +2430,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S7" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:19">
@@ -2483,7 +2483,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S8" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:19">
@@ -2536,7 +2536,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S9" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:19">
@@ -2589,7 +2589,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S10" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:19">
@@ -2642,7 +2642,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S11" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:19">
@@ -2695,7 +2695,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S12" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:19">
@@ -2748,7 +2748,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S13" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:19">
@@ -2801,7 +2801,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S14" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:19">
@@ -2854,7 +2854,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S15" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:19">
@@ -2907,7 +2907,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S16" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:19">
@@ -2960,7 +2960,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S17" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:19">
@@ -3013,7 +3013,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S18" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:19">
@@ -3066,7 +3066,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S19" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:19">
@@ -3119,7 +3119,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S20" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:19">
@@ -3172,7 +3172,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S21" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:19">
@@ -3225,7 +3225,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S22" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:19">
@@ -3278,7 +3278,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S23" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:19">
@@ -3331,7 +3331,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S24" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:19">
@@ -3384,7 +3384,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S25" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:19">
@@ -3437,7 +3437,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S26" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:19">
@@ -3490,7 +3490,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S27" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:19">
@@ -3543,7 +3543,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S28" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:19">
@@ -3596,7 +3596,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S29" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:19">
@@ -3649,7 +3649,7 @@
         <x:v>45842</x:v>
       </x:c>
       <x:c r="S30" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:19">
@@ -3702,7 +3702,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S31" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:19">
@@ -3755,7 +3755,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S32" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062616</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:19">
@@ -3808,7 +3808,7 @@
         <x:v>45843</x:v>
       </x:c>
       <x:c r="S33" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062731</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:19">
@@ -3861,7 +3861,7 @@
         <x:v>45839</x:v>
       </x:c>
       <x:c r="S34" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062731</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:19">
@@ -3914,7 +3914,7 @@
         <x:v>45839</x:v>
       </x:c>
       <x:c r="S35" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062731</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:19">
@@ -3967,7 +3967,7 @@
         <x:v>45839</x:v>
       </x:c>
       <x:c r="S36" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439062731</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:19">
@@ -4020,7 +4020,7 @@
         <x:v>45839</x:v>
       </x:c>
       <x:c r="S37" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:19">
@@ -4073,7 +4073,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S38" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="39" spans="1:19">
@@ -4126,7 +4126,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S39" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="40" spans="1:19">
@@ -4179,7 +4179,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S40" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:19">
@@ -4232,7 +4232,7 @@
         <x:v>45847</x:v>
       </x:c>
       <x:c r="S41" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:19">
@@ -4285,7 +4285,7 @@
         <x:v>45842</x:v>
       </x:c>
       <x:c r="S42" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="43" spans="1:19">
@@ -4338,7 +4338,7 @@
         <x:v>45849</x:v>
       </x:c>
       <x:c r="S43" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="44" spans="1:19">
@@ -4391,7 +4391,7 @@
         <x:v>45842</x:v>
       </x:c>
       <x:c r="S44" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="45" spans="1:19">
@@ -4444,7 +4444,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S45" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="46" spans="1:19">
@@ -4497,7 +4497,7 @@
         <x:v>45839</x:v>
       </x:c>
       <x:c r="S46" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="47" spans="1:19">
@@ -4550,7 +4550,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S47" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:19">
@@ -4603,7 +4603,7 @@
         <x:v>45842</x:v>
       </x:c>
       <x:c r="S48" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="49" spans="1:19">
@@ -4656,7 +4656,7 @@
         <x:v>45849</x:v>
       </x:c>
       <x:c r="S49" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="50" spans="1:19">
@@ -4709,7 +4709,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S50" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="51" spans="1:19">
@@ -4762,7 +4762,7 @@
         <x:v>45842</x:v>
       </x:c>
       <x:c r="S51" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="52" spans="1:19">
@@ -4815,7 +4815,7 @@
         <x:v>45849</x:v>
       </x:c>
       <x:c r="S52" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="53" spans="1:19">
@@ -4868,7 +4868,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S53" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="54" spans="1:19">
@@ -4921,7 +4921,7 @@
         <x:v>45842</x:v>
       </x:c>
       <x:c r="S54" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="55" spans="1:19">
@@ -4974,7 +4974,7 @@
         <x:v>45849</x:v>
       </x:c>
       <x:c r="S55" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="56" spans="1:19">
@@ -5027,7 +5027,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S56" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="57" spans="1:19">
@@ -5080,7 +5080,7 @@
         <x:v>45842</x:v>
       </x:c>
       <x:c r="S57" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="58" spans="1:19">
@@ -5133,7 +5133,7 @@
         <x:v>45849</x:v>
       </x:c>
       <x:c r="S58" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="59" spans="1:19">
@@ -5186,7 +5186,7 @@
         <x:v>45841</x:v>
       </x:c>
       <x:c r="S59" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="60" spans="1:19">
@@ -5239,7 +5239,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S60" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.4439063194</x:v>
       </x:c>
     </x:row>
     <x:row r="61" spans="1:19">
@@ -5292,7 +5292,7 @@
         <x:v>45842</x:v>
       </x:c>
       <x:c r="S61" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="62" spans="1:19">
@@ -5345,7 +5345,7 @@
         <x:v>45849</x:v>
       </x:c>
       <x:c r="S62" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="63" spans="1:19">
@@ -5398,7 +5398,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S63" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="64" spans="1:19">
@@ -5451,7 +5451,7 @@
         <x:v>45842</x:v>
       </x:c>
       <x:c r="S64" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="65" spans="1:19">
@@ -5504,7 +5504,7 @@
         <x:v>45849</x:v>
       </x:c>
       <x:c r="S65" s="3">
-        <x:v>45892.6204811574</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="66" spans="1:19">
@@ -5557,7 +5557,7 @@
         <x:v>45834</x:v>
       </x:c>
       <x:c r="S66" s="3">
-        <x:v>45892.6204811921</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="67" spans="1:19">
@@ -5610,7 +5610,7 @@
         <x:v>45838</x:v>
       </x:c>
       <x:c r="S67" s="3">
-        <x:v>45892.6204811921</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="68" spans="1:19">
@@ -5663,7 +5663,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S68" s="3">
-        <x:v>45892.6204811921</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="69" spans="1:19">
@@ -5716,7 +5716,7 @@
         <x:v>45841</x:v>
       </x:c>
       <x:c r="S69" s="3">
-        <x:v>45892.6204811921</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="70" spans="1:19">
@@ -5769,7 +5769,7 @@
         <x:v>45845</x:v>
       </x:c>
       <x:c r="S70" s="3">
-        <x:v>45892.6204811921</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="71" spans="1:19">
@@ -5822,7 +5822,7 @@
         <x:v>45838</x:v>
       </x:c>
       <x:c r="S71" s="3">
-        <x:v>45892.6204811921</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="72" spans="1:19">
@@ -5875,7 +5875,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S72" s="3">
-        <x:v>45892.6204811921</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="73" spans="1:19">
@@ -5928,7 +5928,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S73" s="3">
-        <x:v>45892.6204811921</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="74" spans="1:19">
@@ -5981,7 +5981,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S74" s="3">
-        <x:v>45892.6204811921</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="75" spans="1:19">
@@ -6034,7 +6034,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S75" s="3">
-        <x:v>45892.6204811921</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="76" spans="1:19">
@@ -6087,7 +6087,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S76" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="77" spans="1:19">
@@ -6140,7 +6140,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S77" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="78" spans="1:19">
@@ -6193,7 +6193,7 @@
         <x:v>45845</x:v>
       </x:c>
       <x:c r="S78" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="79" spans="1:19">
@@ -6246,7 +6246,7 @@
         <x:v>45841</x:v>
       </x:c>
       <x:c r="S79" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="80" spans="1:19">
@@ -6299,7 +6299,7 @@
         <x:v>45839</x:v>
       </x:c>
       <x:c r="S80" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="81" spans="1:19">
@@ -6352,7 +6352,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S81" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="82" spans="1:19">
@@ -6405,7 +6405,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S82" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="83" spans="1:19">
@@ -6458,7 +6458,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S83" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="84" spans="1:19">
@@ -6511,7 +6511,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S84" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="85" spans="1:19">
@@ -6564,7 +6564,7 @@
         <x:v>45847</x:v>
       </x:c>
       <x:c r="S85" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="86" spans="1:19">
@@ -6617,7 +6617,7 @@
         <x:v>45841</x:v>
       </x:c>
       <x:c r="S86" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="87" spans="1:19">
@@ -6670,7 +6670,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S87" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="88" spans="1:19">
@@ -6723,7 +6723,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S88" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="89" spans="1:19">
@@ -6776,7 +6776,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S89" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="90" spans="1:19">
@@ -6829,7 +6829,7 @@
         <x:v>45842</x:v>
       </x:c>
       <x:c r="S90" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="91" spans="1:19">
@@ -6882,7 +6882,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S91" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="92" spans="1:19">
@@ -6935,7 +6935,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S92" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="93" spans="1:19">
@@ -6988,7 +6988,7 @@
         <x:v>45842</x:v>
       </x:c>
       <x:c r="S93" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="94" spans="1:19">
@@ -7041,7 +7041,7 @@
         <x:v>45849</x:v>
       </x:c>
       <x:c r="S94" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="95" spans="1:19">
@@ -7094,7 +7094,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S95" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="96" spans="1:19">
@@ -7147,7 +7147,7 @@
         <x:v>45834</x:v>
       </x:c>
       <x:c r="S96" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="97" spans="1:19">
@@ -7200,7 +7200,7 @@
         <x:v>45834</x:v>
       </x:c>
       <x:c r="S97" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="98" spans="1:19">
@@ -7253,7 +7253,7 @@
         <x:v>45849</x:v>
       </x:c>
       <x:c r="S98" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="99" spans="1:19">
@@ -7306,7 +7306,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S99" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="100" spans="1:19">
@@ -7359,7 +7359,7 @@
         <x:v>45845</x:v>
       </x:c>
       <x:c r="S100" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="101" spans="1:19">
@@ -7412,7 +7412,7 @@
         <x:v>45834</x:v>
       </x:c>
       <x:c r="S101" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="102" spans="1:19">
@@ -7465,7 +7465,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S102" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="103" spans="1:19">
@@ -7518,7 +7518,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S103" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="104" spans="1:19">
@@ -7571,7 +7571,7 @@
         <x:v>45842</x:v>
       </x:c>
       <x:c r="S104" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="105" spans="1:19">
@@ -7624,7 +7624,7 @@
         <x:v>45849</x:v>
       </x:c>
       <x:c r="S105" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="106" spans="1:19">
@@ -7677,7 +7677,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S106" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="107" spans="1:19">
@@ -7730,7 +7730,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S107" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="108" spans="1:19">
@@ -7783,7 +7783,7 @@
         <x:v>45847</x:v>
       </x:c>
       <x:c r="S108" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="109" spans="1:19">
@@ -7836,7 +7836,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S109" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="110" spans="1:19">
@@ -7889,7 +7889,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S110" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="111" spans="1:19">
@@ -7942,7 +7942,7 @@
         <x:v>45842</x:v>
       </x:c>
       <x:c r="S111" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="112" spans="1:19">
@@ -7995,7 +7995,7 @@
         <x:v>45849</x:v>
       </x:c>
       <x:c r="S112" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="113" spans="1:19">
@@ -8048,7 +8048,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S113" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="114" spans="1:19">
@@ -8101,7 +8101,7 @@
         <x:v>45842</x:v>
       </x:c>
       <x:c r="S114" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="115" spans="1:19">
@@ -8154,7 +8154,7 @@
         <x:v>45849</x:v>
       </x:c>
       <x:c r="S115" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="116" spans="1:19">
@@ -8207,7 +8207,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S116" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="117" spans="1:19">
@@ -8260,7 +8260,7 @@
         <x:v>45842</x:v>
       </x:c>
       <x:c r="S117" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="118" spans="1:19">
@@ -8313,7 +8313,7 @@
         <x:v>45849</x:v>
       </x:c>
       <x:c r="S118" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="119" spans="1:19">
@@ -8366,7 +8366,7 @@
         <x:v>45836</x:v>
       </x:c>
       <x:c r="S119" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="120" spans="1:19">
@@ -8419,7 +8419,7 @@
         <x:v>45842</x:v>
       </x:c>
       <x:c r="S120" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.443906331</x:v>
       </x:c>
     </x:row>
     <x:row r="121" spans="1:19">
@@ -8472,7 +8472,7 @@
         <x:v>45849</x:v>
       </x:c>
       <x:c r="S121" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="122" spans="1:19">
@@ -8525,7 +8525,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S122" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="123" spans="1:19">
@@ -8578,7 +8578,7 @@
         <x:v>45850</x:v>
       </x:c>
       <x:c r="S123" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="124" spans="1:19">
@@ -8631,7 +8631,7 @@
         <x:v>45866</x:v>
       </x:c>
       <x:c r="S124" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="125" spans="1:19">
@@ -8684,7 +8684,7 @@
         <x:v>45866</x:v>
       </x:c>
       <x:c r="S125" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="126" spans="1:19">
@@ -8737,7 +8737,7 @@
         <x:v>45866</x:v>
       </x:c>
       <x:c r="S126" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="127" spans="1:19">
@@ -8790,7 +8790,7 @@
         <x:v>45866</x:v>
       </x:c>
       <x:c r="S127" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="128" spans="1:19">
@@ -8843,7 +8843,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S128" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="129" spans="1:19">
@@ -8896,7 +8896,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S129" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="130" spans="1:19">
@@ -8949,7 +8949,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S130" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="131" spans="1:19">
@@ -9002,7 +9002,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S131" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="132" spans="1:19">
@@ -9055,7 +9055,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S132" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="133" spans="1:19">
@@ -9108,7 +9108,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S133" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="134" spans="1:19">
@@ -9161,7 +9161,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S134" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="135" spans="1:19">
@@ -9214,7 +9214,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S135" s="3">
-        <x:v>45892.6204812037</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="136" spans="1:19">
@@ -9267,7 +9267,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S136" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="137" spans="1:19">
@@ -9320,7 +9320,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S137" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="138" spans="1:19">
@@ -9373,7 +9373,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S138" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="139" spans="1:19">
@@ -9426,7 +9426,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S139" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="140" spans="1:19">
@@ -9479,7 +9479,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S140" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="141" spans="1:19">
@@ -9532,7 +9532,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S141" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="142" spans="1:19">
@@ -9585,7 +9585,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S142" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="143" spans="1:19">
@@ -9638,7 +9638,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S143" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="144" spans="1:19">
@@ -9691,7 +9691,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S144" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="145" spans="1:19">
@@ -9744,7 +9744,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S145" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="146" spans="1:19">
@@ -9797,7 +9797,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S146" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="147" spans="1:19">
@@ -9850,7 +9850,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S147" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="148" spans="1:19">
@@ -9903,7 +9903,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S148" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="149" spans="1:19">
@@ -9956,7 +9956,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S149" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="150" spans="1:19">
@@ -10009,7 +10009,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S150" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="151" spans="1:19">
@@ -10062,7 +10062,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S151" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="152" spans="1:19">
@@ -10115,7 +10115,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S152" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="153" spans="1:19">
@@ -10168,7 +10168,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S153" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="154" spans="1:19">
@@ -10221,7 +10221,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S154" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="155" spans="1:19">
@@ -10274,7 +10274,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S155" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="156" spans="1:19">
@@ -10327,7 +10327,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S156" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="157" spans="1:19">
@@ -10380,7 +10380,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S157" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="158" spans="1:19">
@@ -10433,7 +10433,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S158" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="159" spans="1:19">
@@ -10486,7 +10486,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S159" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="160" spans="1:19">
@@ -10539,7 +10539,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S160" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="161" spans="1:19">
@@ -10592,7 +10592,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S161" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="162" spans="1:19">
@@ -10645,7 +10645,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S162" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="163" spans="1:19">
@@ -10698,7 +10698,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S163" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="164" spans="1:19">
@@ -10751,7 +10751,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S164" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="165" spans="1:19">
@@ -10804,7 +10804,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S165" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="166" spans="1:19">
@@ -10857,7 +10857,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S166" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="167" spans="1:19">
@@ -10910,7 +10910,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S167" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="168" spans="1:19">
@@ -10963,7 +10963,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S168" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="169" spans="1:19">
@@ -11016,7 +11016,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S169" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="170" spans="1:19">
@@ -11069,7 +11069,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S170" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="171" spans="1:19">
@@ -11122,7 +11122,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S171" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="172" spans="1:19">
@@ -11175,7 +11175,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S172" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="173" spans="1:19">
@@ -11228,7 +11228,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S173" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="174" spans="1:19">
@@ -11281,7 +11281,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S174" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="175" spans="1:19">
@@ -11334,7 +11334,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S175" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="176" spans="1:19">
@@ -11387,7 +11387,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S176" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="177" spans="1:19">
@@ -11440,7 +11440,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S177" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="178" spans="1:19">
@@ -11493,7 +11493,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S178" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="179" spans="1:19">
@@ -11546,7 +11546,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S179" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="180" spans="1:19">
@@ -11599,7 +11599,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S180" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="181" spans="1:19">
@@ -11652,7 +11652,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S181" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063426</x:v>
       </x:c>
     </x:row>
     <x:row r="182" spans="1:19">
@@ -11705,7 +11705,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S182" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="183" spans="1:19">
@@ -11758,7 +11758,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S183" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="184" spans="1:19">
@@ -11811,7 +11811,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S184" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="185" spans="1:19">
@@ -11864,7 +11864,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S185" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="186" spans="1:19">
@@ -11917,7 +11917,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S186" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="187" spans="1:19">
@@ -11970,7 +11970,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S187" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="188" spans="1:19">
@@ -12023,7 +12023,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S188" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="189" spans="1:19">
@@ -12076,7 +12076,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S189" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="190" spans="1:19">
@@ -12129,7 +12129,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S190" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="191" spans="1:19">
@@ -12182,7 +12182,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S191" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="192" spans="1:19">
@@ -12235,7 +12235,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S192" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="193" spans="1:19">
@@ -12288,7 +12288,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S193" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="194" spans="1:19">
@@ -12341,7 +12341,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S194" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="195" spans="1:19">
@@ -12394,7 +12394,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S195" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="196" spans="1:19">
@@ -12447,7 +12447,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S196" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="197" spans="1:19">
@@ -12500,7 +12500,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S197" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="198" spans="1:19">
@@ -12553,7 +12553,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S198" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="199" spans="1:19">
@@ -12606,7 +12606,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S199" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="200" spans="1:19">
@@ -12659,7 +12659,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S200" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="201" spans="1:19">
@@ -12712,7 +12712,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S201" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="202" spans="1:19">
@@ -12765,7 +12765,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S202" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="203" spans="1:19">
@@ -12818,7 +12818,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S203" s="3">
-        <x:v>45892.6204812153</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="204" spans="1:19">
@@ -12871,7 +12871,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S204" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="205" spans="1:19">
@@ -12924,7 +12924,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S205" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="206" spans="1:19">
@@ -12977,7 +12977,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S206" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="207" spans="1:19">
@@ -13030,7 +13030,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S207" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="208" spans="1:19">
@@ -13083,7 +13083,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S208" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="209" spans="1:19">
@@ -13136,7 +13136,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S209" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="210" spans="1:19">
@@ -13189,7 +13189,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S210" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="211" spans="1:19">
@@ -13242,7 +13242,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S211" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="212" spans="1:19">
@@ -13295,7 +13295,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S212" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="213" spans="1:19">
@@ -13348,7 +13348,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S213" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="214" spans="1:19">
@@ -13401,7 +13401,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S214" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="215" spans="1:19">
@@ -13454,7 +13454,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S215" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="216" spans="1:19">
@@ -13507,7 +13507,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S216" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="217" spans="1:19">
@@ -13560,7 +13560,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S217" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="218" spans="1:19">
@@ -13613,7 +13613,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S218" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="219" spans="1:19">
@@ -13666,7 +13666,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S219" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="220" spans="1:19">
@@ -13719,7 +13719,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S220" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="221" spans="1:19">
@@ -13772,7 +13772,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S221" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="222" spans="1:19">
@@ -13825,7 +13825,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S222" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="223" spans="1:19">
@@ -13878,7 +13878,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S223" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="224" spans="1:19">
@@ -13931,7 +13931,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S224" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="225" spans="1:19">
@@ -13984,7 +13984,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S225" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="226" spans="1:19">
@@ -14037,7 +14037,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S226" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="227" spans="1:19">
@@ -14090,7 +14090,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S227" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="228" spans="1:19">
@@ -14143,7 +14143,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S228" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="229" spans="1:19">
@@ -14196,7 +14196,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S229" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="230" spans="1:19">
@@ -14249,7 +14249,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S230" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="231" spans="1:19">
@@ -14302,7 +14302,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S231" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="232" spans="1:19">
@@ -14355,7 +14355,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S232" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="233" spans="1:19">
@@ -14408,7 +14408,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S233" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="234" spans="1:19">
@@ -14461,7 +14461,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S234" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="235" spans="1:19">
@@ -14514,7 +14514,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S235" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="236" spans="1:19">
@@ -14567,7 +14567,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S236" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="237" spans="1:19">
@@ -14620,7 +14620,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S237" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="238" spans="1:19">
@@ -14673,7 +14673,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S238" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="239" spans="1:19">
@@ -14726,7 +14726,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S239" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="240" spans="1:19">
@@ -14779,7 +14779,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S240" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="241" spans="1:19">
@@ -14832,7 +14832,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S241" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="242" spans="1:19">
@@ -14885,7 +14885,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S242" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="243" spans="1:19">
@@ -14938,7 +14938,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S243" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="244" spans="1:19">
@@ -14991,7 +14991,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S244" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="245" spans="1:19">
@@ -15044,7 +15044,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S245" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063542</x:v>
       </x:c>
     </x:row>
     <x:row r="246" spans="1:19">
@@ -15097,7 +15097,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S246" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="247" spans="1:19">
@@ -15150,7 +15150,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S247" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="248" spans="1:19">
@@ -15203,7 +15203,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S248" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="249" spans="1:19">
@@ -15256,7 +15256,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S249" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="250" spans="1:19">
@@ -15309,7 +15309,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S250" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="251" spans="1:19">
@@ -15362,7 +15362,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S251" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="252" spans="1:19">
@@ -15415,7 +15415,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S252" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="253" spans="1:19">
@@ -15468,7 +15468,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S253" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="254" spans="1:19">
@@ -15521,7 +15521,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S254" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="255" spans="1:19">
@@ -15574,7 +15574,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S255" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="256" spans="1:19">
@@ -15627,7 +15627,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S256" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="257" spans="1:19">
@@ -15680,7 +15680,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S257" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="258" spans="1:19">
@@ -15733,7 +15733,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S258" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="259" spans="1:19">
@@ -15786,7 +15786,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S259" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="260" spans="1:19">
@@ -15839,7 +15839,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S260" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="261" spans="1:19">
@@ -15892,7 +15892,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S261" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="262" spans="1:19">
@@ -15945,7 +15945,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S262" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="263" spans="1:19">
@@ -15998,7 +15998,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S263" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="264" spans="1:19">
@@ -16051,7 +16051,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S264" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="265" spans="1:19">
@@ -16104,7 +16104,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S265" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="266" spans="1:19">
@@ -16157,7 +16157,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S266" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="267" spans="1:19">
@@ -16210,7 +16210,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S267" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="268" spans="1:19">
@@ -16263,7 +16263,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S268" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="269" spans="1:19">
@@ -16316,7 +16316,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S269" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="270" spans="1:19">
@@ -16369,7 +16369,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S270" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="271" spans="1:19">
@@ -16422,7 +16422,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S271" s="3">
-        <x:v>45892.6204812269</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="272" spans="1:19">
@@ -16475,7 +16475,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S272" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="273" spans="1:19">
@@ -16528,7 +16528,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S273" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="274" spans="1:19">
@@ -16581,7 +16581,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S274" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="275" spans="1:19">
@@ -16634,7 +16634,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S275" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="276" spans="1:19">
@@ -16687,7 +16687,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S276" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="277" spans="1:19">
@@ -16740,7 +16740,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S277" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="278" spans="1:19">
@@ -16793,7 +16793,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S278" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="279" spans="1:19">
@@ -16846,7 +16846,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S279" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="280" spans="1:19">
@@ -16899,7 +16899,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S280" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="281" spans="1:19">
@@ -16952,7 +16952,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S281" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="282" spans="1:19">
@@ -17005,7 +17005,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S282" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="283" spans="1:19">
@@ -17058,7 +17058,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S283" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="284" spans="1:19">
@@ -17111,7 +17111,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S284" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="285" spans="1:19">
@@ -17164,7 +17164,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S285" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="286" spans="1:19">
@@ -17217,7 +17217,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S286" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="287" spans="1:19">
@@ -17270,7 +17270,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S287" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="288" spans="1:19">
@@ -17323,7 +17323,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S288" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="289" spans="1:19">
@@ -17376,7 +17376,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S289" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="290" spans="1:19">
@@ -17429,7 +17429,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S290" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="291" spans="1:19">
@@ -17482,7 +17482,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S291" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="292" spans="1:19">
@@ -17535,7 +17535,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S292" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="293" spans="1:19">
@@ -17588,7 +17588,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S293" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="294" spans="1:19">
@@ -17641,7 +17641,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S294" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="295" spans="1:19">
@@ -17694,7 +17694,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S295" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="296" spans="1:19">
@@ -17747,7 +17747,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S296" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="297" spans="1:19">
@@ -17800,7 +17800,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S297" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="298" spans="1:19">
@@ -17853,7 +17853,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S298" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="299" spans="1:19">
@@ -17906,7 +17906,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S299" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="300" spans="1:19">
@@ -17959,7 +17959,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S300" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="301" spans="1:19">
@@ -18012,7 +18012,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S301" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="302" spans="1:19">
@@ -18065,7 +18065,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S302" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="303" spans="1:19">
@@ -18118,7 +18118,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S303" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063657</x:v>
       </x:c>
     </x:row>
     <x:row r="304" spans="1:19">
@@ -18171,7 +18171,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S304" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="305" spans="1:19">
@@ -18224,7 +18224,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S305" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="306" spans="1:19">
@@ -18277,7 +18277,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S306" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="307" spans="1:19">
@@ -18330,7 +18330,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S307" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="308" spans="1:19">
@@ -18383,7 +18383,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S308" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="309" spans="1:19">
@@ -18436,7 +18436,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S309" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="310" spans="1:19">
@@ -18489,7 +18489,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S310" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="311" spans="1:19">
@@ -18542,7 +18542,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S311" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="312" spans="1:19">
@@ -18595,7 +18595,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S312" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="313" spans="1:19">
@@ -18648,7 +18648,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S313" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="314" spans="1:19">
@@ -18701,7 +18701,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S314" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="315" spans="1:19">
@@ -18754,7 +18754,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S315" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="316" spans="1:19">
@@ -18807,7 +18807,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S316" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="317" spans="1:19">
@@ -18860,7 +18860,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S317" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="318" spans="1:19">
@@ -18913,7 +18913,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S318" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="319" spans="1:19">
@@ -18966,7 +18966,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S319" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="320" spans="1:19">
@@ -19019,7 +19019,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S320" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="321" spans="1:19">
@@ -19072,7 +19072,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S321" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="322" spans="1:19">
@@ -19125,7 +19125,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S322" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="323" spans="1:19">
@@ -19178,7 +19178,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S323" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="324" spans="1:19">
@@ -19231,7 +19231,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S324" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="325" spans="1:19">
@@ -19284,7 +19284,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S325" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="326" spans="1:19">
@@ -19337,7 +19337,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S326" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="327" spans="1:19">
@@ -19390,7 +19390,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S327" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="328" spans="1:19">
@@ -19443,7 +19443,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S328" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="329" spans="1:19">
@@ -19496,7 +19496,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S329" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="330" spans="1:19">
@@ -19549,7 +19549,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S330" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="331" spans="1:19">
@@ -19602,7 +19602,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S331" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="332" spans="1:19">
@@ -19655,7 +19655,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S332" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="333" spans="1:19">
@@ -19708,7 +19708,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S333" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="334" spans="1:19">
@@ -19761,7 +19761,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S334" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="335" spans="1:19">
@@ -19814,7 +19814,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S335" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="336" spans="1:19">
@@ -19867,7 +19867,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S336" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="337" spans="1:19">
@@ -19920,7 +19920,7 @@
         <x:v>45835</x:v>
       </x:c>
       <x:c r="S337" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="338" spans="1:19">
@@ -19973,7 +19973,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S338" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="339" spans="1:19">
@@ -20026,7 +20026,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S339" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="340" spans="1:19">
@@ -20079,7 +20079,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S340" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="341" spans="1:19">
@@ -20132,7 +20132,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S341" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="342" spans="1:19">
@@ -20185,7 +20185,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S342" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="343" spans="1:19">
@@ -20238,7 +20238,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S343" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="344" spans="1:19">
@@ -20291,7 +20291,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S344" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
     <x:row r="345" spans="1:19">
@@ -20344,7 +20344,7 @@
         <x:v>45857</x:v>
       </x:c>
       <x:c r="S345" s="3">
-        <x:v>45892.6204812384</x:v>
+        <x:v>45894.4439063773</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>